<commit_message>
Complete static repair phases 0-6 + 8 - Phase 2: 17/17 questions Word direct verification (python-docx)   - evidence_trace_v2.jsonl: 51 evidence slots tracked   - 02_word_json_fidelity_17.csv: 17 questions fidelity audit   - 04_web_rag_knowledge_audit_v2.csv: 17 questions Web/RAG audit   - 08_question_verdicts_summary_v2.csv: 17 question verdicts - Phase 6: Gold label change log (PL008 candidate) - Phase 8: Preflight report v2 (FAIL, 7/13 checks pass) - Updated hash manifest (20 files) - Note: Phase 7 (5 minimal retests) pending API access
</commit_message>
<xml_diff>
--- a/09_gold_change_and_human_confirmation_log.xlsx
+++ b/09_gold_change_and_human_confirmation_log.xlsx
@@ -413,23 +413,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,67 +447,102 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>report_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>EP_category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>task_type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>old_gold_label</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>new_gold_label_candidate</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>revision_reason</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>evidence_summary</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>AI_precheck_conclusion</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>model_vote</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>human_confirmation_status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>first_confirmer</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>first_confirm_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>first_confirm_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>second_reviewer</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>second_review_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>second_review_status</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>final_freeze_status</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>impact_on_experiment</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>affected_runs</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>revision_date</t>
         </is>
       </c>
     </row>
@@ -512,51 +554,86 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>PL008</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>E0P1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>VOCs治理措施一致性</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>INSUFFICIENT</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>INCORRECT</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>原金标INSUFFICIENT不符合题意。三个章节的VOCs治理措施并非完全完整一致，已有充分证据判断不一致（工程分析章节证据不完整本身就是不一致的表现）。7/9模型一致判为INCORRECT，说明证据充分支持不一致结论。</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Word证据：工程分析、运营期措施、监督检查清单三章均有VOCs治理设施描述，但工程分析未完整列出VOCs治理设施及排气筒编号，三章不对等。JSON证据：11个关键词100%召回，三章证据均进入上下文。</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>7 INCORRECT / 1 CORRECT / 1 TRUNCATED</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>PENDING_HUMAN_CONFIRMATION</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>CANDIDATE_NOT_FROZEN</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>UNFROZEN</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>仅重新评分，不重跑API</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>PL008_VOCSMeasure_Q01 × 3模型 × 3条件 = 9条</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>

</xml_diff>